<commit_message>
fix(content): drop the photograph the sheet named but nobody uploaded
The Profesores sheet named mishel_fernandez.jpg, a file that was never in
src/assets/images/teachers and never would be. The importer wrote the name
into academy.json without complaint and the site quietly fell back to her
initials, so nothing anywhere said the reference was dead.

Only the filename goes. Everything else on her row is real and stays: the
styles she teaches, her class, her age and her certification.

With it gone, content/horarios.xlsx imports cleanly for the first time, so
the workflow that rebuilds the site from the workbook can actually run.
</commit_message>
<xml_diff>
--- a/content/horarios.xlsx
+++ b/content/horarios.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="320" uniqueCount="109">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="319" uniqueCount="108">
   <si>
     <t>Dia</t>
   </si>
@@ -260,9 +260,6 @@
   </si>
   <si>
     <t>Salsa, Bachata</t>
-  </si>
-  <si>
-    <t>mishel_fernandez.jpg</t>
   </si>
   <si>
     <t>Giusmary</t>
@@ -727,7 +724,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H55"/>
+  <dimension ref="A1:H16"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -1155,45 +1152,6 @@
         <v>15</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.25"/>
   </sheetData>
   <dataValidations count="8">
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Valor no permitido" error="Elegí una opción de la lista." sqref="A10:A55">
@@ -1222,13 +1180,13 @@
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C36"/>
+  <dimension ref="A1:C17"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -1423,25 +1381,6 @@
         <v>15</v>
       </c>
     </row>
-    <row r="18" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="19" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="20" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="21" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="22" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="23" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="24" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="25" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="26" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="27" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="28" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="29" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="30" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="31" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="32" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="33" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="34" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="35" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="36" spans="2:2" x14ac:dyDescent="0.25"/>
   </sheetData>
   <dataValidations count="2">
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Valor no permitido" error="Elegí una opción de la lista." sqref="B10:B36">
@@ -1452,7 +1391,7 @@
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -1686,9 +1625,6 @@
       <c r="C10" t="s">
         <v>81</v>
       </c>
-      <c r="D10" t="s">
-        <v>82</v>
-      </c>
       <c r="E10" t="s">
         <v>15</v>
       </c>
@@ -1704,7 +1640,7 @@
         <v>12</v>
       </c>
       <c r="B11" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C11" t="s">
         <v>11</v>
@@ -1727,7 +1663,7 @@
         <v>18</v>
       </c>
       <c r="B12" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="C12" t="s">
         <v>17</v>
@@ -1750,7 +1686,7 @@
         <v>23</v>
       </c>
       <c r="B13" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C13" t="s">
         <v>22</v>
@@ -1773,7 +1709,7 @@
         <v>31</v>
       </c>
       <c r="B14" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C14" t="s">
         <v>29</v>
@@ -1796,7 +1732,7 @@
         <v>38</v>
       </c>
       <c r="B15" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C15" t="s">
         <v>37</v>
@@ -1819,7 +1755,7 @@
         <v>44</v>
       </c>
       <c r="B16" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C16" t="s">
         <v>43</v>
@@ -1842,13 +1778,13 @@
         <v>35</v>
       </c>
       <c r="B17" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C17" t="s">
         <v>34</v>
       </c>
       <c r="D17" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="E17" t="s">
         <v>15</v>
@@ -1862,7 +1798,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -1877,10 +1813,10 @@
   <sheetData>
     <row r="1" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>91</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>92</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
@@ -1888,44 +1824,44 @@
         <v>46</v>
       </c>
       <c r="B2" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>93</v>
+      </c>
+      <c r="B3" t="s">
         <v>94</v>
-      </c>
-      <c r="B3" t="s">
-        <v>95</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>95</v>
+      </c>
+      <c r="B4" t="s">
         <v>96</v>
-      </c>
-      <c r="B4" t="s">
-        <v>97</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>97</v>
+      </c>
+      <c r="B5" t="s">
         <v>98</v>
-      </c>
-      <c r="B5" t="s">
-        <v>99</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
+        <v>99</v>
+      </c>
+      <c r="B6" t="s">
         <v>100</v>
-      </c>
-      <c r="B6" t="s">
-        <v>101</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B7" t="s">
         <v>15</v>
@@ -1933,10 +1869,10 @@
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
+        <v>102</v>
+      </c>
+      <c r="B8" t="s">
         <v>103</v>
-      </c>
-      <c r="B8" t="s">
-        <v>104</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
@@ -1944,7 +1880,7 @@
         <v>62</v>
       </c>
       <c r="B9" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
@@ -1952,19 +1888,19 @@
         <v>63</v>
       </c>
       <c r="B10" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
+        <v>106</v>
+      </c>
+      <c r="B11" t="s">
         <v>107</v>
-      </c>
-      <c r="B11" t="s">
-        <v>108</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(content): a placeholder teacher for the Sexy Style classes
Both Sexy Style classes had an empty Profesor cell, and no teacher listed
the genre. They now name "Por confirmar", a row of its own in the
Profesores sheet, to be renamed once the real teacher is known.

The workbook also takes the dropdown fix from the template: its Genero and
Profesor lists read the sheets, so the real name can be chosen when it
arrives instead of being refused by Excel.
</commit_message>
<xml_diff>
--- a/content/horarios.xlsx
+++ b/content/horarios.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="319" uniqueCount="108">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="322" uniqueCount="109">
   <si>
     <t>Dia</t>
   </si>
@@ -98,6 +98,9 @@
   </si>
   <si>
     <t>Sexy Style</t>
+  </si>
+  <si>
+    <t>Por confirmar</t>
   </si>
   <si>
     <t>21:00</t>
@@ -854,7 +857,7 @@
         <v>27</v>
       </c>
       <c r="E5" t="s">
-        <v>15</v>
+        <v>28</v>
       </c>
       <c r="F5" t="s">
         <v>13</v>
@@ -874,13 +877,13 @@
         <v>26</v>
       </c>
       <c r="C6" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D6" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="E6" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="F6" t="s">
         <v>24</v>
@@ -897,19 +900,19 @@
         <v>25</v>
       </c>
       <c r="B7" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C7" t="s">
         <v>21</v>
       </c>
       <c r="D7" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="E7" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="F7" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="G7" t="s">
         <v>14</v>
@@ -920,7 +923,7 @@
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B8" t="s">
         <v>9</v>
@@ -946,7 +949,7 @@
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B9" t="s">
         <v>10</v>
@@ -955,10 +958,10 @@
         <v>16</v>
       </c>
       <c r="D9" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="E9" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="F9" t="s">
         <v>19</v>
@@ -972,7 +975,7 @@
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B10" t="s">
         <v>10</v>
@@ -984,7 +987,7 @@
         <v>27</v>
       </c>
       <c r="E10" t="s">
-        <v>15</v>
+        <v>28</v>
       </c>
       <c r="F10" t="s">
         <v>13</v>
@@ -998,19 +1001,19 @@
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B11" t="s">
         <v>26</v>
       </c>
       <c r="C11" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D11" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="E11" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="F11" t="s">
         <v>24</v>
@@ -1024,22 +1027,22 @@
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B12" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C12" t="s">
         <v>21</v>
       </c>
       <c r="D12" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="E12" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="F12" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="G12" t="s">
         <v>14</v>
@@ -1050,13 +1053,13 @@
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B13" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C13" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="D13" t="s">
         <v>22</v>
@@ -1071,12 +1074,12 @@
         <v>14</v>
       </c>
       <c r="H13" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B14" t="s">
         <v>10</v>
@@ -1085,10 +1088,10 @@
         <v>16</v>
       </c>
       <c r="D14" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="E14" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="F14" t="s">
         <v>19</v>
@@ -1102,7 +1105,7 @@
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B15" t="s">
         <v>16</v>
@@ -1111,7 +1114,7 @@
         <v>21</v>
       </c>
       <c r="D15" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="E15" t="s">
         <v>15</v>
@@ -1128,7 +1131,7 @@
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B16" t="s">
         <v>16</v>
@@ -1137,7 +1140,7 @@
         <v>21</v>
       </c>
       <c r="D16" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="E16" t="s">
         <v>15</v>
@@ -1154,28 +1157,28 @@
     </row>
   </sheetData>
   <dataValidations count="8">
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Valor no permitido" error="Elegí una opción de la lista." sqref="A10:A55">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Valor no permitido" error="Elige una opción de la lista." sqref="A10:A55">
       <formula1>"Lunes,Martes,Miércoles,Jueves,Viernes,Sábado,Domingo"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Valor no permitido" error="Elegí una opción de la lista." sqref="A2:A55">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Valor no permitido" error="Elige una opción de la lista." sqref="A2:A55">
       <formula1>"Lunes,Martes,Miércoles,Jueves,Viernes,Sábado,Domingo"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Valor no permitido" error="Elegí una opción de la lista." sqref="D10:D55">
-      <formula1>"Salsa,Bachata,Jazz,Latin Urban,Ladies,Ballet,Urban Style,Mambo,Body Movement,Urban Dance,Sexy Style,Sexy Power,Comercial Dance,Heels,Reggaeton,Ensayo Elenco"</formula1>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Valor no permitido" error="Elige una opción de la lista." sqref="D10:D55">
+      <formula1>Generos!$A$2:$A$36</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Valor no permitido" error="Elegí una opción de la lista." sqref="D2:D55">
-      <formula1>"Salsa,Bachata,Jazz,Latin Urban,Ladies,Ballet,Urban Style,Mambo,Body Movement,Urban Dance,Sexy Style,Sexy Power,Comercial Dance,Heels,Reggaeton,Ensayo Elenco"</formula1>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Valor no permitido" error="Elige una opción de la lista." sqref="D2:D55">
+      <formula1>Generos!$A$2:$A$36</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Valor no permitido" error="Elegí una opción de la lista." sqref="E10:E55">
-      <formula1>"Izquierdo,Joan,Martinez,Kike,Pedro,Stefanie,Mary,Estrella,Mishel Fernández,Giusmary Sosa,Vannia Valdivia,Edson Cabanillas,Kenneth Ocaña,Omar López,Anthony Sevillano,Gonzalo Povis"</formula1>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Valor no permitido" error="Elige una opción de la lista." sqref="E10:E55">
+      <formula1>Profesores!$A$2:$A$37</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Valor no permitido" error="Elegí una opción de la lista." sqref="E2:E55">
-      <formula1>"Izquierdo,Joan,Martinez,Kike,Pedro,Stefanie,Mary,Estrella,Mishel Fernández,Giusmary Sosa,Vannia Valdivia,Edson Cabanillas,Kenneth Ocaña,Omar López,Anthony Sevillano,Gonzalo Povis"</formula1>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Valor no permitido" error="Elige una opción de la lista." sqref="E2:E55">
+      <formula1>Profesores!$A$2:$A$37</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Valor no permitido" error="Elegí una opción de la lista." sqref="F10:F55">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Valor no permitido" error="Elige una opción de la lista." sqref="F10:F55">
       <formula1>"Principiantes,Básico,Intermedio,Avanzado,All levels"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Valor no permitido" error="Elegí una opción de la lista." sqref="F2:F55">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Valor no permitido" error="Elige una opción de la lista." sqref="F2:F55">
       <formula1>"Principiantes,Básico,Intermedio,Avanzado,All levels"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1186,7 +1189,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C17"/>
+  <dimension ref="A1:C18"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -1196,21 +1199,21 @@
   <sheetData>
     <row r="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B2" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C2" t="s">
         <v>15</v>
@@ -1218,10 +1221,10 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B3" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C3" t="s">
         <v>15</v>
@@ -1229,10 +1232,10 @@
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>51</v>
+      </c>
+      <c r="B4" t="s">
         <v>50</v>
-      </c>
-      <c r="B4" t="s">
-        <v>49</v>
       </c>
       <c r="C4" t="s">
         <v>15</v>
@@ -1240,10 +1243,10 @@
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B5" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C5" t="s">
         <v>15</v>
@@ -1251,10 +1254,10 @@
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B6" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C6" t="s">
         <v>15</v>
@@ -1262,10 +1265,10 @@
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B7" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C7" t="s">
         <v>15</v>
@@ -1273,10 +1276,10 @@
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B8" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C8" t="s">
         <v>15</v>
@@ -1284,10 +1287,10 @@
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B9" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C9" t="s">
         <v>15</v>
@@ -1295,10 +1298,10 @@
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B10" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C10" t="s">
         <v>15</v>
@@ -1309,7 +1312,7 @@
         <v>11</v>
       </c>
       <c r="B11" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C11" t="s">
         <v>15</v>
@@ -1320,7 +1323,7 @@
         <v>27</v>
       </c>
       <c r="B12" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C12" t="s">
         <v>15</v>
@@ -1331,7 +1334,7 @@
         <v>17</v>
       </c>
       <c r="B13" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C13" t="s">
         <v>15</v>
@@ -1339,10 +1342,10 @@
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B14" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C14" t="s">
         <v>15</v>
@@ -1353,7 +1356,7 @@
         <v>22</v>
       </c>
       <c r="B15" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C15" t="s">
         <v>15</v>
@@ -1361,10 +1364,10 @@
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B16" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C16" t="s">
         <v>15</v>
@@ -1372,21 +1375,22 @@
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B17" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C17" t="s">
         <v>15</v>
       </c>
     </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Valor no permitido" error="Elegí una opción de la lista." sqref="B10:B36">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Valor no permitido" error="Elige una opción de la lista." sqref="B10:B36">
       <formula1>"Clase,Ensayo"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Valor no permitido" error="Elegí una opción de la lista." sqref="B2:B36">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Valor no permitido" error="Elige una opción de la lista." sqref="B2:B36">
       <formula1>"Clase,Ensayo"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1397,7 +1401,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G17"/>
+  <dimension ref="A1:G19"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
@@ -1410,39 +1414,39 @@
   <sheetData>
     <row r="1" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B2" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E2" t="s">
         <v>15</v>
@@ -1456,16 +1460,16 @@
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B3" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C3" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D3" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E3" t="s">
         <v>15</v>
@@ -1479,16 +1483,16 @@
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B4" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C4" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D4" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="E4" t="s">
         <v>15</v>
@@ -1502,16 +1506,16 @@
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B5" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C5" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D5" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="E5" t="s">
         <v>15</v>
@@ -1525,16 +1529,16 @@
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B6" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C6" t="s">
         <v>15</v>
       </c>
       <c r="D6" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="E6" t="s">
         <v>15</v>
@@ -1548,16 +1552,16 @@
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B7" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C7" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D7" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="E7" t="s">
         <v>15</v>
@@ -1571,16 +1575,16 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B8" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C8" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D8" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="E8" t="s">
         <v>15</v>
@@ -1594,16 +1598,16 @@
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B9" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C9" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D9" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="E9" t="s">
         <v>15</v>
@@ -1617,13 +1621,13 @@
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B10" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C10" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="E10" t="s">
         <v>15</v>
@@ -1640,7 +1644,7 @@
         <v>12</v>
       </c>
       <c r="B11" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C11" t="s">
         <v>11</v>
@@ -1663,7 +1667,7 @@
         <v>18</v>
       </c>
       <c r="B12" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C12" t="s">
         <v>17</v>
@@ -1686,7 +1690,7 @@
         <v>23</v>
       </c>
       <c r="B13" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C13" t="s">
         <v>22</v>
@@ -1706,13 +1710,13 @@
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B14" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C14" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D14" t="s">
         <v>15</v>
@@ -1729,13 +1733,13 @@
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
+        <v>39</v>
+      </c>
+      <c r="B15" t="s">
+        <v>87</v>
+      </c>
+      <c r="C15" t="s">
         <v>38</v>
-      </c>
-      <c r="B15" t="s">
-        <v>86</v>
-      </c>
-      <c r="C15" t="s">
-        <v>37</v>
       </c>
       <c r="D15" t="s">
         <v>15</v>
@@ -1752,13 +1756,13 @@
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
+        <v>45</v>
+      </c>
+      <c r="B16" t="s">
+        <v>88</v>
+      </c>
+      <c r="C16" t="s">
         <v>44</v>
-      </c>
-      <c r="B16" t="s">
-        <v>87</v>
-      </c>
-      <c r="C16" t="s">
-        <v>43</v>
       </c>
       <c r="D16" t="s">
         <v>15</v>
@@ -1775,16 +1779,16 @@
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
+        <v>36</v>
+      </c>
+      <c r="B17" t="s">
+        <v>89</v>
+      </c>
+      <c r="C17" t="s">
         <v>35</v>
       </c>
-      <c r="B17" t="s">
-        <v>88</v>
-      </c>
-      <c r="C17" t="s">
-        <v>34</v>
-      </c>
       <c r="D17" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="E17" t="s">
         <v>15</v>
@@ -1796,6 +1800,18 @@
         <v>15</v>
       </c>
     </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>28</v>
+      </c>
+      <c r="B18" t="s">
+        <v>28</v>
+      </c>
+      <c r="C18" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -1813,55 +1829,55 @@
   <sheetData>
     <row r="1" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B2" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="B3" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B4" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="B5" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B6" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B7" t="s">
         <v>15</v>
@@ -1869,34 +1885,34 @@
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="B8" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B9" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B10" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B11" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
     </row>
   </sheetData>

</xml_diff>